<commit_message>
feat: add for n=8
</commit_message>
<xml_diff>
--- a/CS4221 Project Results.xlsx
+++ b/CS4221 Project Results.xlsx
@@ -7,7 +7,7 @@
     <sheet name="Archived Data" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Archived Data'!$A$1:$O$309</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Archived Data'!$A$1:$O$327</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -1427,7 +1427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O309"/>
+  <dimension ref="A1:O327"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -15092,7 +15092,7 @@
     </row>
     <row r="291">
       <c r="A291" t="n">
-        <v>20</v>
+        <v>1</v>
       </c>
       <c r="B291" t="n">
         <v>8</v>
@@ -15101,45 +15101,45 @@
         <v>1016</v>
       </c>
       <c r="D291" t="n">
-        <v>0.01968503937007874</v>
+        <v>0.000984251968503937</v>
       </c>
       <c r="E291" t="n">
-        <v>12.1494</v>
+        <v>0.9812</v>
       </c>
       <c r="F291" t="n">
-        <v>0.01195807086614173</v>
+        <v>0.0009657480314960629</v>
       </c>
       <c r="G291" t="n">
         <v>30000</v>
       </c>
       <c r="H291" t="n">
-        <v>954</v>
+        <v>15</v>
       </c>
       <c r="I291" t="n">
-        <v>266</v>
+        <v>72</v>
       </c>
       <c r="J291" t="n">
-        <v>28762</v>
+        <v>18748</v>
       </c>
       <c r="K291" t="n">
-        <v>18</v>
+        <v>11165</v>
       </c>
       <c r="L291" t="n">
-        <v>0.0318</v>
+        <v>0.0005</v>
       </c>
       <c r="M291" t="n">
-        <v>0.008866666666666667</v>
+        <v>0.0024</v>
       </c>
       <c r="N291" t="n">
-        <v>0.9587333333333333</v>
+        <v>0.6249333333333333</v>
       </c>
       <c r="O291" t="n">
-        <v>0.0005999999999999999</v>
+        <v>0.3721666666666666</v>
       </c>
     </row>
     <row r="292">
       <c r="A292" t="n">
-        <v>40</v>
+        <v>20</v>
       </c>
       <c r="B292" t="n">
         <v>8</v>
@@ -15148,45 +15148,45 @@
         <v>1016</v>
       </c>
       <c r="D292" t="n">
-        <v>0.03937007874015748</v>
+        <v>0.01968503937007874</v>
       </c>
       <c r="E292" t="n">
-        <v>13.909783</v>
+        <v>12.1494</v>
       </c>
       <c r="F292" t="n">
-        <v>0.0136907312992126</v>
+        <v>0.01195807086614173</v>
       </c>
       <c r="G292" t="n">
         <v>30000</v>
       </c>
       <c r="H292" t="n">
-        <v>499</v>
+        <v>954</v>
       </c>
       <c r="I292" t="n">
-        <v>6</v>
+        <v>266</v>
       </c>
       <c r="J292" t="n">
-        <v>29107</v>
+        <v>28762</v>
       </c>
       <c r="K292" t="n">
-        <v>388</v>
+        <v>18</v>
       </c>
       <c r="L292" t="n">
-        <v>0.01663333333333333</v>
+        <v>0.0318</v>
       </c>
       <c r="M292" t="n">
-        <v>0.0002</v>
+        <v>0.008866666666666667</v>
       </c>
       <c r="N292" t="n">
-        <v>0.9702333333333333</v>
+        <v>0.9587333333333333</v>
       </c>
       <c r="O292" t="n">
-        <v>0.01293333333333333</v>
+        <v>0.0005999999999999999</v>
       </c>
     </row>
     <row r="293">
       <c r="A293" t="n">
-        <v>51</v>
+        <v>40</v>
       </c>
       <c r="B293" t="n">
         <v>8</v>
@@ -15195,45 +15195,45 @@
         <v>1016</v>
       </c>
       <c r="D293" t="n">
-        <v>0.05019685039370079</v>
+        <v>0.03937007874015748</v>
       </c>
       <c r="E293" t="n">
-        <v>13.641033</v>
+        <v>13.909783</v>
       </c>
       <c r="F293" t="n">
-        <v>0.01342621358267717</v>
+        <v>0.0136907312992126</v>
       </c>
       <c r="G293" t="n">
         <v>30000</v>
       </c>
       <c r="H293" t="n">
-        <v>471</v>
+        <v>499</v>
       </c>
       <c r="I293" t="n">
         <v>6</v>
       </c>
       <c r="J293" t="n">
-        <v>28444</v>
+        <v>29107</v>
       </c>
       <c r="K293" t="n">
-        <v>1079</v>
+        <v>388</v>
       </c>
       <c r="L293" t="n">
-        <v>0.0157</v>
+        <v>0.01663333333333333</v>
       </c>
       <c r="M293" t="n">
         <v>0.0002</v>
       </c>
       <c r="N293" t="n">
-        <v>0.9481333333333334</v>
+        <v>0.9702333333333333</v>
       </c>
       <c r="O293" t="n">
-        <v>0.03596666666666667</v>
+        <v>0.01293333333333333</v>
       </c>
     </row>
     <row r="294">
       <c r="A294" t="n">
-        <v>60</v>
+        <v>51</v>
       </c>
       <c r="B294" t="n">
         <v>8</v>
@@ -15242,45 +15242,45 @@
         <v>1016</v>
       </c>
       <c r="D294" t="n">
-        <v>0.05905511811023622</v>
+        <v>0.05019685039370079</v>
       </c>
       <c r="E294" t="n">
-        <v>13.32325</v>
+        <v>13.641033</v>
       </c>
       <c r="F294" t="n">
-        <v>0.01311343503937008</v>
+        <v>0.01342621358267717</v>
       </c>
       <c r="G294" t="n">
         <v>30000</v>
       </c>
       <c r="H294" t="n">
-        <v>504</v>
+        <v>471</v>
       </c>
       <c r="I294" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="J294" t="n">
-        <v>27595</v>
+        <v>28444</v>
       </c>
       <c r="K294" t="n">
-        <v>1900</v>
+        <v>1079</v>
       </c>
       <c r="L294" t="n">
-        <v>0.0168</v>
+        <v>0.0157</v>
       </c>
       <c r="M294" t="n">
-        <v>3.333333333333333e-05</v>
+        <v>0.0002</v>
       </c>
       <c r="N294" t="n">
-        <v>0.9198333333333333</v>
+        <v>0.9481333333333334</v>
       </c>
       <c r="O294" t="n">
-        <v>0.06333333333333334</v>
+        <v>0.03596666666666667</v>
       </c>
     </row>
     <row r="295">
       <c r="A295" t="n">
-        <v>100</v>
+        <v>60</v>
       </c>
       <c r="B295" t="n">
         <v>8</v>
@@ -15289,45 +15289,45 @@
         <v>1016</v>
       </c>
       <c r="D295" t="n">
-        <v>0.09842519685039371</v>
+        <v>0.05905511811023622</v>
       </c>
       <c r="E295" t="n">
-        <v>11.7137</v>
+        <v>13.32325</v>
       </c>
       <c r="F295" t="n">
-        <v>0.01152923228346457</v>
+        <v>0.01311343503937008</v>
       </c>
       <c r="G295" t="n">
         <v>30000</v>
       </c>
       <c r="H295" t="n">
-        <v>905</v>
+        <v>504</v>
       </c>
       <c r="I295" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J295" t="n">
-        <v>20647</v>
+        <v>27595</v>
       </c>
       <c r="K295" t="n">
-        <v>8448</v>
+        <v>1900</v>
       </c>
       <c r="L295" t="n">
-        <v>0.03016666666666667</v>
+        <v>0.0168</v>
       </c>
       <c r="M295" t="n">
-        <v>0</v>
+        <v>3.333333333333333e-05</v>
       </c>
       <c r="N295" t="n">
-        <v>0.6882333333333334</v>
+        <v>0.9198333333333333</v>
       </c>
       <c r="O295" t="n">
-        <v>0.2816</v>
+        <v>0.06333333333333334</v>
       </c>
     </row>
     <row r="296">
       <c r="A296" t="n">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="B296" t="n">
         <v>8</v>
@@ -15336,45 +15336,45 @@
         <v>1016</v>
       </c>
       <c r="D296" t="n">
-        <v>0.1003937007874016</v>
+        <v>0.09842519685039371</v>
       </c>
       <c r="E296" t="n">
-        <v>11.794033</v>
+        <v>11.7137</v>
       </c>
       <c r="F296" t="n">
-        <v>0.01160830019685039</v>
+        <v>0.01152923228346457</v>
       </c>
       <c r="G296" t="n">
         <v>30000</v>
       </c>
       <c r="H296" t="n">
-        <v>942</v>
+        <v>905</v>
       </c>
       <c r="I296" t="n">
         <v>0</v>
       </c>
       <c r="J296" t="n">
-        <v>20220</v>
+        <v>20647</v>
       </c>
       <c r="K296" t="n">
-        <v>8838</v>
+        <v>8448</v>
       </c>
       <c r="L296" t="n">
-        <v>0.0314</v>
+        <v>0.03016666666666667</v>
       </c>
       <c r="M296" t="n">
         <v>0</v>
       </c>
       <c r="N296" t="n">
-        <v>0.674</v>
+        <v>0.6882333333333334</v>
       </c>
       <c r="O296" t="n">
-        <v>0.2946</v>
+        <v>0.2816</v>
       </c>
     </row>
     <row r="297">
       <c r="A297" t="n">
-        <v>203</v>
+        <v>102</v>
       </c>
       <c r="B297" t="n">
         <v>8</v>
@@ -15383,608 +15383,1454 @@
         <v>1016</v>
       </c>
       <c r="D297" t="n">
-        <v>0.1998031496062992</v>
+        <v>0.1003937007874016</v>
       </c>
       <c r="E297" t="n">
-        <v>9.705033</v>
+        <v>11.794033</v>
       </c>
       <c r="F297" t="n">
-        <v>0.009552197834645669</v>
+        <v>0.01160830019685039</v>
       </c>
       <c r="G297" t="n">
         <v>30000</v>
       </c>
       <c r="H297" t="n">
-        <v>1291</v>
+        <v>942</v>
       </c>
       <c r="I297" t="n">
         <v>0</v>
       </c>
       <c r="J297" t="n">
-        <v>3883</v>
+        <v>20220</v>
       </c>
       <c r="K297" t="n">
-        <v>24826</v>
+        <v>8838</v>
       </c>
       <c r="L297" t="n">
-        <v>0.04303333333333333</v>
+        <v>0.0314</v>
       </c>
       <c r="M297" t="n">
         <v>0</v>
       </c>
       <c r="N297" t="n">
-        <v>0.1294333333333333</v>
+        <v>0.674</v>
       </c>
       <c r="O297" t="n">
-        <v>0.8275333333333333</v>
+        <v>0.2946</v>
       </c>
     </row>
     <row r="298">
       <c r="A298" t="n">
-        <v>20</v>
+        <v>152</v>
       </c>
       <c r="B298" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C298" t="n">
-        <v>2295</v>
+        <v>1016</v>
       </c>
       <c r="D298" t="n">
-        <v>0.008714596949891068</v>
+        <v>0.1496062992125984</v>
       </c>
       <c r="E298" t="n">
-        <v>14.223367</v>
+        <v>10.538025</v>
       </c>
       <c r="F298" t="n">
-        <v>0.006197545533769063</v>
+        <v>0.0103720718503937</v>
       </c>
       <c r="G298" t="n">
         <v>30000</v>
       </c>
       <c r="H298" t="n">
-        <v>349</v>
+        <v>1466</v>
       </c>
       <c r="I298" t="n">
-        <v>181</v>
+        <v>0</v>
       </c>
       <c r="J298" t="n">
-        <v>29470</v>
+        <v>10269</v>
       </c>
       <c r="K298" t="n">
-        <v>0</v>
+        <v>18265</v>
       </c>
       <c r="L298" t="n">
-        <v>0.01163333333333333</v>
+        <v>0.04886666666666667</v>
       </c>
       <c r="M298" t="n">
-        <v>0.006033333333333333</v>
+        <v>0</v>
       </c>
       <c r="N298" t="n">
-        <v>0.9823333333333333</v>
+        <v>0.3423</v>
       </c>
       <c r="O298" t="n">
-        <v>0</v>
+        <v>0.6088333333333333</v>
       </c>
     </row>
     <row r="299">
       <c r="A299" t="n">
-        <v>40</v>
+        <v>203</v>
       </c>
       <c r="B299" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C299" t="n">
-        <v>2295</v>
+        <v>1016</v>
       </c>
       <c r="D299" t="n">
-        <v>0.01742919389978214</v>
+        <v>0.1998031496062992</v>
       </c>
       <c r="E299" t="n">
-        <v>18.5792</v>
+        <v>9.705033</v>
       </c>
       <c r="F299" t="n">
-        <v>0.008095511982570806</v>
+        <v>0.009552197834645669</v>
       </c>
       <c r="G299" t="n">
         <v>30000</v>
       </c>
       <c r="H299" t="n">
-        <v>154</v>
+        <v>1291</v>
       </c>
       <c r="I299" t="n">
-        <v>18</v>
+        <v>0</v>
       </c>
       <c r="J299" t="n">
-        <v>29816</v>
+        <v>3883</v>
       </c>
       <c r="K299" t="n">
-        <v>12</v>
+        <v>24826</v>
       </c>
       <c r="L299" t="n">
-        <v>0.005133333333333333</v>
+        <v>0.04303333333333333</v>
       </c>
       <c r="M299" t="n">
-        <v>0.0005999999999999999</v>
+        <v>0</v>
       </c>
       <c r="N299" t="n">
-        <v>0.9938666666666667</v>
+        <v>0.1294333333333333</v>
       </c>
       <c r="O299" t="n">
-        <v>0.0004</v>
+        <v>0.8275333333333333</v>
       </c>
     </row>
     <row r="300">
       <c r="A300" t="n">
-        <v>60</v>
+        <v>254</v>
       </c>
       <c r="B300" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C300" t="n">
-        <v>2295</v>
+        <v>1016</v>
       </c>
       <c r="D300" t="n">
-        <v>0.0261437908496732</v>
+        <v>0.25</v>
       </c>
       <c r="E300" t="n">
-        <v>19.173983</v>
+        <v>9.444732999999999</v>
       </c>
       <c r="F300" t="n">
-        <v>0.008354676688453159</v>
+        <v>0.009295997047244094</v>
       </c>
       <c r="G300" t="n">
         <v>30000</v>
       </c>
       <c r="H300" t="n">
-        <v>82</v>
+        <v>866</v>
       </c>
       <c r="I300" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J300" t="n">
-        <v>29844</v>
+        <v>1146</v>
       </c>
       <c r="K300" t="n">
-        <v>73</v>
+        <v>27988</v>
       </c>
       <c r="L300" t="n">
-        <v>0.002733333333333333</v>
+        <v>0.02886666666666667</v>
       </c>
       <c r="M300" t="n">
-        <v>3.333333333333333e-05</v>
+        <v>0</v>
       </c>
       <c r="N300" t="n">
-        <v>0.9948</v>
+        <v>0.0382</v>
       </c>
       <c r="O300" t="n">
-        <v>0.002433333333333333</v>
+        <v>0.9329333333333333</v>
       </c>
     </row>
     <row r="301">
       <c r="A301" t="n">
-        <v>92</v>
+        <v>305</v>
       </c>
       <c r="B301" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C301" t="n">
-        <v>2295</v>
+        <v>1016</v>
       </c>
       <c r="D301" t="n">
-        <v>0.04008714596949891</v>
+        <v>0.3001968503937008</v>
       </c>
       <c r="E301" t="n">
-        <v>18.0652</v>
+        <v>9.384024999999999</v>
       </c>
       <c r="F301" t="n">
-        <v>0.007871546840958607</v>
+        <v>0.009236245078740157</v>
       </c>
       <c r="G301" t="n">
-        <v>20000</v>
+        <v>30000</v>
       </c>
       <c r="H301" t="n">
-        <v>65</v>
+        <v>406</v>
       </c>
       <c r="I301" t="n">
         <v>0</v>
       </c>
       <c r="J301" t="n">
-        <v>19614</v>
+        <v>236</v>
       </c>
       <c r="K301" t="n">
-        <v>321</v>
+        <v>29358</v>
       </c>
       <c r="L301" t="n">
-        <v>0.00325</v>
+        <v>0.01353333333333333</v>
       </c>
       <c r="M301" t="n">
         <v>0</v>
       </c>
       <c r="N301" t="n">
-        <v>0.9807</v>
+        <v>0.007866666666666666</v>
       </c>
       <c r="O301" t="n">
-        <v>0.01605</v>
+        <v>0.9786</v>
       </c>
     </row>
     <row r="302">
       <c r="A302" t="n">
-        <v>100</v>
+        <v>356</v>
       </c>
       <c r="B302" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C302" t="n">
-        <v>2295</v>
+        <v>1016</v>
       </c>
       <c r="D302" t="n">
-        <v>0.04357298474945534</v>
+        <v>0.3503937007874016</v>
       </c>
       <c r="E302" t="n">
-        <v>17.6535</v>
+        <v>9.25855</v>
       </c>
       <c r="F302" t="n">
-        <v>0.007692156862745099</v>
+        <v>0.009112746062992125</v>
       </c>
       <c r="G302" t="n">
         <v>30000</v>
       </c>
       <c r="H302" t="n">
-        <v>135</v>
+        <v>149</v>
       </c>
       <c r="I302" t="n">
         <v>0</v>
       </c>
       <c r="J302" t="n">
-        <v>29185</v>
+        <v>48</v>
       </c>
       <c r="K302" t="n">
-        <v>680</v>
+        <v>29803</v>
       </c>
       <c r="L302" t="n">
-        <v>0.0045</v>
+        <v>0.004966666666666667</v>
       </c>
       <c r="M302" t="n">
         <v>0</v>
       </c>
       <c r="N302" t="n">
-        <v>0.9728333333333333</v>
+        <v>0.0016</v>
       </c>
       <c r="O302" t="n">
-        <v>0.02266666666666667</v>
+        <v>0.9934333333333333</v>
       </c>
     </row>
     <row r="303">
       <c r="A303" t="n">
-        <v>20</v>
+        <v>406</v>
       </c>
       <c r="B303" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="C303" t="n">
-        <v>5110</v>
+        <v>1016</v>
       </c>
       <c r="D303" t="n">
-        <v>0.003913894324853229</v>
+        <v>0.3996062992125984</v>
       </c>
       <c r="E303" t="n">
-        <v>15.884733</v>
+        <v>10.104767</v>
       </c>
       <c r="F303" t="n">
-        <v>0.003108558317025441</v>
+        <v>0.009945636811023622</v>
       </c>
       <c r="G303" t="n">
         <v>30000</v>
       </c>
       <c r="H303" t="n">
-        <v>142</v>
+        <v>46</v>
       </c>
       <c r="I303" t="n">
-        <v>93</v>
+        <v>0</v>
       </c>
       <c r="J303" t="n">
-        <v>29765</v>
+        <v>14</v>
       </c>
       <c r="K303" t="n">
-        <v>0</v>
+        <v>29940</v>
       </c>
       <c r="L303" t="n">
-        <v>0.004733333333333333</v>
+        <v>0.001533333333333333</v>
       </c>
       <c r="M303" t="n">
-        <v>0.0031</v>
+        <v>0</v>
       </c>
       <c r="N303" t="n">
-        <v>0.9921666666666666</v>
+        <v>0.0004666666666666667</v>
       </c>
       <c r="O303" t="n">
-        <v>0</v>
+        <v>0.998</v>
       </c>
     </row>
     <row r="304">
       <c r="A304" t="n">
-        <v>40</v>
+        <v>457</v>
       </c>
       <c r="B304" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="C304" t="n">
-        <v>5110</v>
+        <v>1016</v>
       </c>
       <c r="D304" t="n">
-        <v>0.007827788649706457</v>
+        <v>0.4498031496062992</v>
       </c>
       <c r="E304" t="n">
-        <v>23.273367</v>
+        <v>10.204933</v>
       </c>
       <c r="F304" t="n">
-        <v>0.004554474951076321</v>
+        <v>0.01004422539370079</v>
       </c>
       <c r="G304" t="n">
         <v>30000</v>
       </c>
       <c r="H304" t="n">
-        <v>41</v>
+        <v>15</v>
       </c>
       <c r="I304" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="J304" t="n">
-        <v>29954</v>
+        <v>0</v>
       </c>
       <c r="K304" t="n">
-        <v>0</v>
+        <v>29985</v>
       </c>
       <c r="L304" t="n">
-        <v>0.001366666666666667</v>
+        <v>0.0005</v>
       </c>
       <c r="M304" t="n">
-        <v>0.0001666666666666667</v>
+        <v>0</v>
       </c>
       <c r="N304" t="n">
-        <v>0.9984666666666666</v>
+        <v>0</v>
       </c>
       <c r="O304" t="n">
-        <v>0</v>
+        <v>0.9995000000000001</v>
       </c>
     </row>
     <row r="305">
       <c r="A305" t="n">
-        <v>60</v>
+        <v>508</v>
       </c>
       <c r="B305" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="C305" t="n">
-        <v>5110</v>
+        <v>1016</v>
       </c>
       <c r="D305" t="n">
-        <v>0.01174168297455969</v>
+        <v>0.5</v>
       </c>
       <c r="E305" t="n">
-        <v>25.9887</v>
+        <v>9.5761</v>
       </c>
       <c r="F305" t="n">
-        <v>0.005085851272015656</v>
+        <v>0.009425295275590552</v>
       </c>
       <c r="G305" t="n">
         <v>30000</v>
       </c>
       <c r="H305" t="n">
-        <v>15</v>
+        <v>1</v>
       </c>
       <c r="I305" t="n">
         <v>0</v>
       </c>
       <c r="J305" t="n">
-        <v>29985</v>
+        <v>0</v>
       </c>
       <c r="K305" t="n">
-        <v>0</v>
+        <v>29999</v>
       </c>
       <c r="L305" t="n">
-        <v>0.0005</v>
+        <v>3.333333333333333e-05</v>
       </c>
       <c r="M305" t="n">
         <v>0</v>
       </c>
       <c r="N305" t="n">
-        <v>0.9995000000000001</v>
+        <v>0</v>
       </c>
       <c r="O305" t="n">
-        <v>0</v>
+        <v>0.9999666666666667</v>
       </c>
     </row>
     <row r="306">
       <c r="A306" t="n">
-        <v>102</v>
+        <v>559</v>
       </c>
       <c r="B306" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="C306" t="n">
-        <v>5110</v>
+        <v>1016</v>
       </c>
       <c r="D306" t="n">
-        <v>0.01996086105675147</v>
+        <v>0.5501968503937008</v>
       </c>
       <c r="E306" t="n">
-        <v>26.4037</v>
+        <v>9.705966999999999</v>
       </c>
       <c r="F306" t="n">
-        <v>0.005167064579256361</v>
+        <v>0.009553117125984251</v>
       </c>
       <c r="G306" t="n">
         <v>30000</v>
       </c>
       <c r="H306" t="n">
-        <v>19</v>
+        <v>0</v>
       </c>
       <c r="I306" t="n">
         <v>0</v>
       </c>
       <c r="J306" t="n">
-        <v>29961</v>
+        <v>0</v>
       </c>
       <c r="K306" t="n">
-        <v>20</v>
+        <v>30000</v>
       </c>
       <c r="L306" t="n">
-        <v>0.0006333333333333333</v>
+        <v>0</v>
       </c>
       <c r="M306" t="n">
         <v>0</v>
       </c>
       <c r="N306" t="n">
-        <v>0.9987</v>
+        <v>0</v>
       </c>
       <c r="O306" t="n">
-        <v>0.0006666666666666666</v>
+        <v>1</v>
       </c>
     </row>
     <row r="307">
       <c r="A307" t="n">
-        <v>20</v>
+        <v>610</v>
       </c>
       <c r="B307" t="n">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="C307" t="n">
-        <v>11253</v>
+        <v>1016</v>
       </c>
       <c r="D307" t="n">
-        <v>0.001777303830089754</v>
+        <v>0.6003937007874016</v>
       </c>
       <c r="E307" t="n">
-        <v>17.141133</v>
+        <v>9.609467</v>
       </c>
       <c r="F307" t="n">
-        <v>0.001523250066648894</v>
+        <v>0.009458136811023622</v>
       </c>
       <c r="G307" t="n">
         <v>30000</v>
       </c>
       <c r="H307" t="n">
-        <v>38</v>
+        <v>0</v>
       </c>
       <c r="I307" t="n">
-        <v>51</v>
+        <v>0</v>
       </c>
       <c r="J307" t="n">
-        <v>29911</v>
+        <v>0</v>
       </c>
       <c r="K307" t="n">
-        <v>0</v>
+        <v>30000</v>
       </c>
       <c r="L307" t="n">
-        <v>0.001266666666666667</v>
+        <v>0</v>
       </c>
       <c r="M307" t="n">
-        <v>0.0017</v>
+        <v>0</v>
       </c>
       <c r="N307" t="n">
-        <v>0.9970333333333333</v>
+        <v>0</v>
       </c>
       <c r="O307" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="308">
       <c r="A308" t="n">
-        <v>20</v>
+        <v>660</v>
       </c>
       <c r="B308" t="n">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="C308" t="n">
-        <v>24564</v>
+        <v>1016</v>
       </c>
       <c r="D308" t="n">
-        <v>0.0008141996417521576</v>
+        <v>0.6496062992125984</v>
       </c>
       <c r="E308" t="n">
-        <v>18.048667</v>
+        <v>8.504533</v>
       </c>
       <c r="F308" t="n">
-        <v>0.0007347609102751994</v>
+        <v>0.008370603346456694</v>
       </c>
       <c r="G308" t="n">
         <v>30000</v>
       </c>
       <c r="H308" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="I308" t="n">
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="J308" t="n">
-        <v>29983</v>
+        <v>0</v>
       </c>
       <c r="K308" t="n">
-        <v>0</v>
+        <v>30000</v>
       </c>
       <c r="L308" t="n">
-        <v>0.0002</v>
+        <v>0</v>
       </c>
       <c r="M308" t="n">
-        <v>0.0003666666666666667</v>
+        <v>0</v>
       </c>
       <c r="N308" t="n">
-        <v>0.9994333333333333</v>
+        <v>0</v>
       </c>
       <c r="O308" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="309">
       <c r="A309" t="n">
+        <v>711</v>
+      </c>
+      <c r="B309" t="n">
+        <v>8</v>
+      </c>
+      <c r="C309" t="n">
+        <v>1016</v>
+      </c>
+      <c r="D309" t="n">
+        <v>0.6998031496062992</v>
+      </c>
+      <c r="E309" t="n">
+        <v>9.446899999999999</v>
+      </c>
+      <c r="F309" t="n">
+        <v>0.009298129921259841</v>
+      </c>
+      <c r="G309" t="n">
+        <v>30000</v>
+      </c>
+      <c r="H309" t="n">
+        <v>0</v>
+      </c>
+      <c r="I309" t="n">
+        <v>0</v>
+      </c>
+      <c r="J309" t="n">
+        <v>0</v>
+      </c>
+      <c r="K309" t="n">
+        <v>30000</v>
+      </c>
+      <c r="L309" t="n">
+        <v>0</v>
+      </c>
+      <c r="M309" t="n">
+        <v>0</v>
+      </c>
+      <c r="N309" t="n">
+        <v>0</v>
+      </c>
+      <c r="O309" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="310">
+      <c r="A310" t="n">
+        <v>762</v>
+      </c>
+      <c r="B310" t="n">
+        <v>8</v>
+      </c>
+      <c r="C310" t="n">
+        <v>1016</v>
+      </c>
+      <c r="D310" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="E310" t="n">
+        <v>9.958</v>
+      </c>
+      <c r="F310" t="n">
+        <v>0.009801181102362205</v>
+      </c>
+      <c r="G310" t="n">
+        <v>30000</v>
+      </c>
+      <c r="H310" t="n">
+        <v>0</v>
+      </c>
+      <c r="I310" t="n">
+        <v>0</v>
+      </c>
+      <c r="J310" t="n">
+        <v>0</v>
+      </c>
+      <c r="K310" t="n">
+        <v>30000</v>
+      </c>
+      <c r="L310" t="n">
+        <v>0</v>
+      </c>
+      <c r="M310" t="n">
+        <v>0</v>
+      </c>
+      <c r="N310" t="n">
+        <v>0</v>
+      </c>
+      <c r="O310" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="311">
+      <c r="A311" t="n">
+        <v>813</v>
+      </c>
+      <c r="B311" t="n">
+        <v>8</v>
+      </c>
+      <c r="C311" t="n">
+        <v>1016</v>
+      </c>
+      <c r="D311" t="n">
+        <v>0.8001968503937008</v>
+      </c>
+      <c r="E311" t="n">
+        <v>9.076533</v>
+      </c>
+      <c r="F311" t="n">
+        <v>0.008933595472440945</v>
+      </c>
+      <c r="G311" t="n">
+        <v>30000</v>
+      </c>
+      <c r="H311" t="n">
+        <v>0</v>
+      </c>
+      <c r="I311" t="n">
+        <v>0</v>
+      </c>
+      <c r="J311" t="n">
+        <v>0</v>
+      </c>
+      <c r="K311" t="n">
+        <v>30000</v>
+      </c>
+      <c r="L311" t="n">
+        <v>0</v>
+      </c>
+      <c r="M311" t="n">
+        <v>0</v>
+      </c>
+      <c r="N311" t="n">
+        <v>0</v>
+      </c>
+      <c r="O311" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="312">
+      <c r="A312" t="n">
+        <v>864</v>
+      </c>
+      <c r="B312" t="n">
+        <v>8</v>
+      </c>
+      <c r="C312" t="n">
+        <v>1016</v>
+      </c>
+      <c r="D312" t="n">
+        <v>0.8503937007874016</v>
+      </c>
+      <c r="E312" t="n">
+        <v>9.183267000000001</v>
+      </c>
+      <c r="F312" t="n">
+        <v>0.009038648622047245</v>
+      </c>
+      <c r="G312" t="n">
+        <v>30000</v>
+      </c>
+      <c r="H312" t="n">
+        <v>0</v>
+      </c>
+      <c r="I312" t="n">
+        <v>0</v>
+      </c>
+      <c r="J312" t="n">
+        <v>0</v>
+      </c>
+      <c r="K312" t="n">
+        <v>30000</v>
+      </c>
+      <c r="L312" t="n">
+        <v>0</v>
+      </c>
+      <c r="M312" t="n">
+        <v>0</v>
+      </c>
+      <c r="N312" t="n">
+        <v>0</v>
+      </c>
+      <c r="O312" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="313">
+      <c r="A313" t="n">
+        <v>914</v>
+      </c>
+      <c r="B313" t="n">
+        <v>8</v>
+      </c>
+      <c r="C313" t="n">
+        <v>1016</v>
+      </c>
+      <c r="D313" t="n">
+        <v>0.8996062992125984</v>
+      </c>
+      <c r="E313" t="n">
+        <v>9.891299999999999</v>
+      </c>
+      <c r="F313" t="n">
+        <v>0.009735531496062991</v>
+      </c>
+      <c r="G313" t="n">
+        <v>30000</v>
+      </c>
+      <c r="H313" t="n">
+        <v>0</v>
+      </c>
+      <c r="I313" t="n">
+        <v>0</v>
+      </c>
+      <c r="J313" t="n">
+        <v>0</v>
+      </c>
+      <c r="K313" t="n">
+        <v>30000</v>
+      </c>
+      <c r="L313" t="n">
+        <v>0</v>
+      </c>
+      <c r="M313" t="n">
+        <v>0</v>
+      </c>
+      <c r="N313" t="n">
+        <v>0</v>
+      </c>
+      <c r="O313" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="314">
+      <c r="A314" t="n">
+        <v>965</v>
+      </c>
+      <c r="B314" t="n">
+        <v>8</v>
+      </c>
+      <c r="C314" t="n">
+        <v>1016</v>
+      </c>
+      <c r="D314" t="n">
+        <v>0.9498031496062992</v>
+      </c>
+      <c r="E314" t="n">
+        <v>10</v>
+      </c>
+      <c r="F314" t="n">
+        <v>0.00984251968503937</v>
+      </c>
+      <c r="G314" t="n">
+        <v>30000</v>
+      </c>
+      <c r="H314" t="n">
+        <v>0</v>
+      </c>
+      <c r="I314" t="n">
+        <v>0</v>
+      </c>
+      <c r="J314" t="n">
+        <v>0</v>
+      </c>
+      <c r="K314" t="n">
+        <v>30000</v>
+      </c>
+      <c r="L314" t="n">
+        <v>0</v>
+      </c>
+      <c r="M314" t="n">
+        <v>0</v>
+      </c>
+      <c r="N314" t="n">
+        <v>0</v>
+      </c>
+      <c r="O314" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="315">
+      <c r="A315" t="n">
+        <v>1016</v>
+      </c>
+      <c r="B315" t="n">
+        <v>8</v>
+      </c>
+      <c r="C315" t="n">
+        <v>1016</v>
+      </c>
+      <c r="D315" t="n">
+        <v>1</v>
+      </c>
+      <c r="E315" t="n">
+        <v>10</v>
+      </c>
+      <c r="F315" t="n">
+        <v>0.00984251968503937</v>
+      </c>
+      <c r="G315" t="n">
+        <v>30000</v>
+      </c>
+      <c r="H315" t="n">
+        <v>0</v>
+      </c>
+      <c r="I315" t="n">
+        <v>0</v>
+      </c>
+      <c r="J315" t="n">
+        <v>0</v>
+      </c>
+      <c r="K315" t="n">
+        <v>30000</v>
+      </c>
+      <c r="L315" t="n">
+        <v>0</v>
+      </c>
+      <c r="M315" t="n">
+        <v>0</v>
+      </c>
+      <c r="N315" t="n">
+        <v>0</v>
+      </c>
+      <c r="O315" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="316">
+      <c r="A316" t="n">
         <v>20</v>
       </c>
-      <c r="B309" t="n">
+      <c r="B316" t="n">
+        <v>9</v>
+      </c>
+      <c r="C316" t="n">
+        <v>2295</v>
+      </c>
+      <c r="D316" t="n">
+        <v>0.008714596949891068</v>
+      </c>
+      <c r="E316" t="n">
+        <v>14.223367</v>
+      </c>
+      <c r="F316" t="n">
+        <v>0.006197545533769063</v>
+      </c>
+      <c r="G316" t="n">
+        <v>30000</v>
+      </c>
+      <c r="H316" t="n">
+        <v>349</v>
+      </c>
+      <c r="I316" t="n">
+        <v>181</v>
+      </c>
+      <c r="J316" t="n">
+        <v>29470</v>
+      </c>
+      <c r="K316" t="n">
+        <v>0</v>
+      </c>
+      <c r="L316" t="n">
+        <v>0.01163333333333333</v>
+      </c>
+      <c r="M316" t="n">
+        <v>0.006033333333333333</v>
+      </c>
+      <c r="N316" t="n">
+        <v>0.9823333333333333</v>
+      </c>
+      <c r="O316" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="317">
+      <c r="A317" t="n">
+        <v>40</v>
+      </c>
+      <c r="B317" t="n">
+        <v>9</v>
+      </c>
+      <c r="C317" t="n">
+        <v>2295</v>
+      </c>
+      <c r="D317" t="n">
+        <v>0.01742919389978214</v>
+      </c>
+      <c r="E317" t="n">
+        <v>18.5792</v>
+      </c>
+      <c r="F317" t="n">
+        <v>0.008095511982570806</v>
+      </c>
+      <c r="G317" t="n">
+        <v>30000</v>
+      </c>
+      <c r="H317" t="n">
+        <v>154</v>
+      </c>
+      <c r="I317" t="n">
+        <v>18</v>
+      </c>
+      <c r="J317" t="n">
+        <v>29816</v>
+      </c>
+      <c r="K317" t="n">
+        <v>12</v>
+      </c>
+      <c r="L317" t="n">
+        <v>0.005133333333333333</v>
+      </c>
+      <c r="M317" t="n">
+        <v>0.0005999999999999999</v>
+      </c>
+      <c r="N317" t="n">
+        <v>0.9938666666666667</v>
+      </c>
+      <c r="O317" t="n">
+        <v>0.0004</v>
+      </c>
+    </row>
+    <row r="318">
+      <c r="A318" t="n">
+        <v>60</v>
+      </c>
+      <c r="B318" t="n">
+        <v>9</v>
+      </c>
+      <c r="C318" t="n">
+        <v>2295</v>
+      </c>
+      <c r="D318" t="n">
+        <v>0.0261437908496732</v>
+      </c>
+      <c r="E318" t="n">
+        <v>19.173983</v>
+      </c>
+      <c r="F318" t="n">
+        <v>0.008354676688453159</v>
+      </c>
+      <c r="G318" t="n">
+        <v>30000</v>
+      </c>
+      <c r="H318" t="n">
+        <v>82</v>
+      </c>
+      <c r="I318" t="n">
+        <v>1</v>
+      </c>
+      <c r="J318" t="n">
+        <v>29844</v>
+      </c>
+      <c r="K318" t="n">
+        <v>73</v>
+      </c>
+      <c r="L318" t="n">
+        <v>0.002733333333333333</v>
+      </c>
+      <c r="M318" t="n">
+        <v>3.333333333333333e-05</v>
+      </c>
+      <c r="N318" t="n">
+        <v>0.9948</v>
+      </c>
+      <c r="O318" t="n">
+        <v>0.002433333333333333</v>
+      </c>
+    </row>
+    <row r="319">
+      <c r="A319" t="n">
+        <v>92</v>
+      </c>
+      <c r="B319" t="n">
+        <v>9</v>
+      </c>
+      <c r="C319" t="n">
+        <v>2295</v>
+      </c>
+      <c r="D319" t="n">
+        <v>0.04008714596949891</v>
+      </c>
+      <c r="E319" t="n">
+        <v>18.0652</v>
+      </c>
+      <c r="F319" t="n">
+        <v>0.007871546840958607</v>
+      </c>
+      <c r="G319" t="n">
+        <v>20000</v>
+      </c>
+      <c r="H319" t="n">
+        <v>65</v>
+      </c>
+      <c r="I319" t="n">
+        <v>0</v>
+      </c>
+      <c r="J319" t="n">
+        <v>19614</v>
+      </c>
+      <c r="K319" t="n">
+        <v>321</v>
+      </c>
+      <c r="L319" t="n">
+        <v>0.00325</v>
+      </c>
+      <c r="M319" t="n">
+        <v>0</v>
+      </c>
+      <c r="N319" t="n">
+        <v>0.9807</v>
+      </c>
+      <c r="O319" t="n">
+        <v>0.01605</v>
+      </c>
+    </row>
+    <row r="320">
+      <c r="A320" t="n">
+        <v>100</v>
+      </c>
+      <c r="B320" t="n">
+        <v>9</v>
+      </c>
+      <c r="C320" t="n">
+        <v>2295</v>
+      </c>
+      <c r="D320" t="n">
+        <v>0.04357298474945534</v>
+      </c>
+      <c r="E320" t="n">
+        <v>17.6535</v>
+      </c>
+      <c r="F320" t="n">
+        <v>0.007692156862745099</v>
+      </c>
+      <c r="G320" t="n">
+        <v>30000</v>
+      </c>
+      <c r="H320" t="n">
+        <v>135</v>
+      </c>
+      <c r="I320" t="n">
+        <v>0</v>
+      </c>
+      <c r="J320" t="n">
+        <v>29185</v>
+      </c>
+      <c r="K320" t="n">
+        <v>680</v>
+      </c>
+      <c r="L320" t="n">
+        <v>0.0045</v>
+      </c>
+      <c r="M320" t="n">
+        <v>0</v>
+      </c>
+      <c r="N320" t="n">
+        <v>0.9728333333333333</v>
+      </c>
+      <c r="O320" t="n">
+        <v>0.02266666666666667</v>
+      </c>
+    </row>
+    <row r="321">
+      <c r="A321" t="n">
+        <v>20</v>
+      </c>
+      <c r="B321" t="n">
+        <v>10</v>
+      </c>
+      <c r="C321" t="n">
+        <v>5110</v>
+      </c>
+      <c r="D321" t="n">
+        <v>0.003913894324853229</v>
+      </c>
+      <c r="E321" t="n">
+        <v>15.884733</v>
+      </c>
+      <c r="F321" t="n">
+        <v>0.003108558317025441</v>
+      </c>
+      <c r="G321" t="n">
+        <v>30000</v>
+      </c>
+      <c r="H321" t="n">
+        <v>142</v>
+      </c>
+      <c r="I321" t="n">
+        <v>93</v>
+      </c>
+      <c r="J321" t="n">
+        <v>29765</v>
+      </c>
+      <c r="K321" t="n">
+        <v>0</v>
+      </c>
+      <c r="L321" t="n">
+        <v>0.004733333333333333</v>
+      </c>
+      <c r="M321" t="n">
+        <v>0.0031</v>
+      </c>
+      <c r="N321" t="n">
+        <v>0.9921666666666666</v>
+      </c>
+      <c r="O321" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="322">
+      <c r="A322" t="n">
+        <v>40</v>
+      </c>
+      <c r="B322" t="n">
+        <v>10</v>
+      </c>
+      <c r="C322" t="n">
+        <v>5110</v>
+      </c>
+      <c r="D322" t="n">
+        <v>0.007827788649706457</v>
+      </c>
+      <c r="E322" t="n">
+        <v>23.273367</v>
+      </c>
+      <c r="F322" t="n">
+        <v>0.004554474951076321</v>
+      </c>
+      <c r="G322" t="n">
+        <v>30000</v>
+      </c>
+      <c r="H322" t="n">
+        <v>41</v>
+      </c>
+      <c r="I322" t="n">
+        <v>5</v>
+      </c>
+      <c r="J322" t="n">
+        <v>29954</v>
+      </c>
+      <c r="K322" t="n">
+        <v>0</v>
+      </c>
+      <c r="L322" t="n">
+        <v>0.001366666666666667</v>
+      </c>
+      <c r="M322" t="n">
+        <v>0.0001666666666666667</v>
+      </c>
+      <c r="N322" t="n">
+        <v>0.9984666666666666</v>
+      </c>
+      <c r="O322" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="323">
+      <c r="A323" t="n">
+        <v>60</v>
+      </c>
+      <c r="B323" t="n">
+        <v>10</v>
+      </c>
+      <c r="C323" t="n">
+        <v>5110</v>
+      </c>
+      <c r="D323" t="n">
+        <v>0.01174168297455969</v>
+      </c>
+      <c r="E323" t="n">
+        <v>25.9887</v>
+      </c>
+      <c r="F323" t="n">
+        <v>0.005085851272015656</v>
+      </c>
+      <c r="G323" t="n">
+        <v>30000</v>
+      </c>
+      <c r="H323" t="n">
+        <v>15</v>
+      </c>
+      <c r="I323" t="n">
+        <v>0</v>
+      </c>
+      <c r="J323" t="n">
+        <v>29985</v>
+      </c>
+      <c r="K323" t="n">
+        <v>0</v>
+      </c>
+      <c r="L323" t="n">
+        <v>0.0005</v>
+      </c>
+      <c r="M323" t="n">
+        <v>0</v>
+      </c>
+      <c r="N323" t="n">
+        <v>0.9995000000000001</v>
+      </c>
+      <c r="O323" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="324">
+      <c r="A324" t="n">
+        <v>102</v>
+      </c>
+      <c r="B324" t="n">
+        <v>10</v>
+      </c>
+      <c r="C324" t="n">
+        <v>5110</v>
+      </c>
+      <c r="D324" t="n">
+        <v>0.01996086105675147</v>
+      </c>
+      <c r="E324" t="n">
+        <v>26.4037</v>
+      </c>
+      <c r="F324" t="n">
+        <v>0.005167064579256361</v>
+      </c>
+      <c r="G324" t="n">
+        <v>30000</v>
+      </c>
+      <c r="H324" t="n">
+        <v>19</v>
+      </c>
+      <c r="I324" t="n">
+        <v>0</v>
+      </c>
+      <c r="J324" t="n">
+        <v>29961</v>
+      </c>
+      <c r="K324" t="n">
+        <v>20</v>
+      </c>
+      <c r="L324" t="n">
+        <v>0.0006333333333333333</v>
+      </c>
+      <c r="M324" t="n">
+        <v>0</v>
+      </c>
+      <c r="N324" t="n">
+        <v>0.9987</v>
+      </c>
+      <c r="O324" t="n">
+        <v>0.0006666666666666666</v>
+      </c>
+    </row>
+    <row r="325">
+      <c r="A325" t="n">
+        <v>20</v>
+      </c>
+      <c r="B325" t="n">
+        <v>11</v>
+      </c>
+      <c r="C325" t="n">
+        <v>11253</v>
+      </c>
+      <c r="D325" t="n">
+        <v>0.001777303830089754</v>
+      </c>
+      <c r="E325" t="n">
+        <v>17.141133</v>
+      </c>
+      <c r="F325" t="n">
+        <v>0.001523250066648894</v>
+      </c>
+      <c r="G325" t="n">
+        <v>30000</v>
+      </c>
+      <c r="H325" t="n">
+        <v>38</v>
+      </c>
+      <c r="I325" t="n">
+        <v>51</v>
+      </c>
+      <c r="J325" t="n">
+        <v>29911</v>
+      </c>
+      <c r="K325" t="n">
+        <v>0</v>
+      </c>
+      <c r="L325" t="n">
+        <v>0.001266666666666667</v>
+      </c>
+      <c r="M325" t="n">
+        <v>0.0017</v>
+      </c>
+      <c r="N325" t="n">
+        <v>0.9970333333333333</v>
+      </c>
+      <c r="O325" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="326">
+      <c r="A326" t="n">
+        <v>20</v>
+      </c>
+      <c r="B326" t="n">
+        <v>12</v>
+      </c>
+      <c r="C326" t="n">
+        <v>24564</v>
+      </c>
+      <c r="D326" t="n">
+        <v>0.0008141996417521576</v>
+      </c>
+      <c r="E326" t="n">
+        <v>18.048667</v>
+      </c>
+      <c r="F326" t="n">
+        <v>0.0007347609102751994</v>
+      </c>
+      <c r="G326" t="n">
+        <v>30000</v>
+      </c>
+      <c r="H326" t="n">
+        <v>6</v>
+      </c>
+      <c r="I326" t="n">
+        <v>11</v>
+      </c>
+      <c r="J326" t="n">
+        <v>29983</v>
+      </c>
+      <c r="K326" t="n">
+        <v>0</v>
+      </c>
+      <c r="L326" t="n">
+        <v>0.0002</v>
+      </c>
+      <c r="M326" t="n">
+        <v>0.0003666666666666667</v>
+      </c>
+      <c r="N326" t="n">
+        <v>0.9994333333333333</v>
+      </c>
+      <c r="O326" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="327">
+      <c r="A327" t="n">
+        <v>20</v>
+      </c>
+      <c r="B327" t="n">
         <v>13</v>
       </c>
-      <c r="C309" t="n">
+      <c r="C327" t="n">
         <v>53235</v>
       </c>
-      <c r="D309" t="n">
+      <c r="D327" t="n">
         <v>0.0003756926833849911</v>
       </c>
-      <c r="E309" t="n">
+      <c r="E327" t="n">
         <v>18.6665</v>
       </c>
-      <c r="F309" t="n">
+      <c r="F327" t="n">
         <v>0.0003506433737202968</v>
       </c>
-      <c r="G309" t="n">
-        <v>30000</v>
-      </c>
-      <c r="H309" t="n">
+      <c r="G327" t="n">
+        <v>30000</v>
+      </c>
+      <c r="H327" t="n">
         <v>7</v>
       </c>
-      <c r="I309" t="n">
+      <c r="I327" t="n">
         <v>5</v>
       </c>
-      <c r="J309" t="n">
+      <c r="J327" t="n">
         <v>29988</v>
       </c>
-      <c r="K309" t="n">
-        <v>0</v>
-      </c>
-      <c r="L309" t="n">
+      <c r="K327" t="n">
+        <v>0</v>
+      </c>
+      <c r="L327" t="n">
         <v>0.0002333333333333333</v>
       </c>
-      <c r="M309" t="n">
+      <c r="M327" t="n">
         <v>0.0001666666666666667</v>
       </c>
-      <c r="N309" t="n">
+      <c r="N327" t="n">
         <v>0.9996</v>
       </c>
-      <c r="O309" t="n">
+      <c r="O327" t="n">
         <v>0</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:O309"/>
+  <autoFilter ref="A1:O327"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: restrict graphs from n=4 to 8
</commit_message>
<xml_diff>
--- a/CS4221 Project Results.xlsx
+++ b/CS4221 Project Results.xlsx
@@ -7,7 +7,7 @@
     <sheet name="Archived Data" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Archived Data'!$A$1:$O$327</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Archived Data'!$A$1:$O$315</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -1427,7 +1427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O327"/>
+  <dimension ref="A1:O315"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -16265,572 +16265,8 @@
         <v>1</v>
       </c>
     </row>
-    <row r="316">
-      <c r="A316" t="n">
-        <v>20</v>
-      </c>
-      <c r="B316" t="n">
-        <v>9</v>
-      </c>
-      <c r="C316" t="n">
-        <v>2295</v>
-      </c>
-      <c r="D316" t="n">
-        <v>0.008714596949891068</v>
-      </c>
-      <c r="E316" t="n">
-        <v>14.223367</v>
-      </c>
-      <c r="F316" t="n">
-        <v>0.006197545533769063</v>
-      </c>
-      <c r="G316" t="n">
-        <v>30000</v>
-      </c>
-      <c r="H316" t="n">
-        <v>349</v>
-      </c>
-      <c r="I316" t="n">
-        <v>181</v>
-      </c>
-      <c r="J316" t="n">
-        <v>29470</v>
-      </c>
-      <c r="K316" t="n">
-        <v>0</v>
-      </c>
-      <c r="L316" t="n">
-        <v>0.01163333333333333</v>
-      </c>
-      <c r="M316" t="n">
-        <v>0.006033333333333333</v>
-      </c>
-      <c r="N316" t="n">
-        <v>0.9823333333333333</v>
-      </c>
-      <c r="O316" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="317">
-      <c r="A317" t="n">
-        <v>40</v>
-      </c>
-      <c r="B317" t="n">
-        <v>9</v>
-      </c>
-      <c r="C317" t="n">
-        <v>2295</v>
-      </c>
-      <c r="D317" t="n">
-        <v>0.01742919389978214</v>
-      </c>
-      <c r="E317" t="n">
-        <v>18.5792</v>
-      </c>
-      <c r="F317" t="n">
-        <v>0.008095511982570806</v>
-      </c>
-      <c r="G317" t="n">
-        <v>30000</v>
-      </c>
-      <c r="H317" t="n">
-        <v>154</v>
-      </c>
-      <c r="I317" t="n">
-        <v>18</v>
-      </c>
-      <c r="J317" t="n">
-        <v>29816</v>
-      </c>
-      <c r="K317" t="n">
-        <v>12</v>
-      </c>
-      <c r="L317" t="n">
-        <v>0.005133333333333333</v>
-      </c>
-      <c r="M317" t="n">
-        <v>0.0005999999999999999</v>
-      </c>
-      <c r="N317" t="n">
-        <v>0.9938666666666667</v>
-      </c>
-      <c r="O317" t="n">
-        <v>0.0004</v>
-      </c>
-    </row>
-    <row r="318">
-      <c r="A318" t="n">
-        <v>60</v>
-      </c>
-      <c r="B318" t="n">
-        <v>9</v>
-      </c>
-      <c r="C318" t="n">
-        <v>2295</v>
-      </c>
-      <c r="D318" t="n">
-        <v>0.0261437908496732</v>
-      </c>
-      <c r="E318" t="n">
-        <v>19.173983</v>
-      </c>
-      <c r="F318" t="n">
-        <v>0.008354676688453159</v>
-      </c>
-      <c r="G318" t="n">
-        <v>30000</v>
-      </c>
-      <c r="H318" t="n">
-        <v>82</v>
-      </c>
-      <c r="I318" t="n">
-        <v>1</v>
-      </c>
-      <c r="J318" t="n">
-        <v>29844</v>
-      </c>
-      <c r="K318" t="n">
-        <v>73</v>
-      </c>
-      <c r="L318" t="n">
-        <v>0.002733333333333333</v>
-      </c>
-      <c r="M318" t="n">
-        <v>3.333333333333333e-05</v>
-      </c>
-      <c r="N318" t="n">
-        <v>0.9948</v>
-      </c>
-      <c r="O318" t="n">
-        <v>0.002433333333333333</v>
-      </c>
-    </row>
-    <row r="319">
-      <c r="A319" t="n">
-        <v>92</v>
-      </c>
-      <c r="B319" t="n">
-        <v>9</v>
-      </c>
-      <c r="C319" t="n">
-        <v>2295</v>
-      </c>
-      <c r="D319" t="n">
-        <v>0.04008714596949891</v>
-      </c>
-      <c r="E319" t="n">
-        <v>18.0652</v>
-      </c>
-      <c r="F319" t="n">
-        <v>0.007871546840958607</v>
-      </c>
-      <c r="G319" t="n">
-        <v>20000</v>
-      </c>
-      <c r="H319" t="n">
-        <v>65</v>
-      </c>
-      <c r="I319" t="n">
-        <v>0</v>
-      </c>
-      <c r="J319" t="n">
-        <v>19614</v>
-      </c>
-      <c r="K319" t="n">
-        <v>321</v>
-      </c>
-      <c r="L319" t="n">
-        <v>0.00325</v>
-      </c>
-      <c r="M319" t="n">
-        <v>0</v>
-      </c>
-      <c r="N319" t="n">
-        <v>0.9807</v>
-      </c>
-      <c r="O319" t="n">
-        <v>0.01605</v>
-      </c>
-    </row>
-    <row r="320">
-      <c r="A320" t="n">
-        <v>100</v>
-      </c>
-      <c r="B320" t="n">
-        <v>9</v>
-      </c>
-      <c r="C320" t="n">
-        <v>2295</v>
-      </c>
-      <c r="D320" t="n">
-        <v>0.04357298474945534</v>
-      </c>
-      <c r="E320" t="n">
-        <v>17.6535</v>
-      </c>
-      <c r="F320" t="n">
-        <v>0.007692156862745099</v>
-      </c>
-      <c r="G320" t="n">
-        <v>30000</v>
-      </c>
-      <c r="H320" t="n">
-        <v>135</v>
-      </c>
-      <c r="I320" t="n">
-        <v>0</v>
-      </c>
-      <c r="J320" t="n">
-        <v>29185</v>
-      </c>
-      <c r="K320" t="n">
-        <v>680</v>
-      </c>
-      <c r="L320" t="n">
-        <v>0.0045</v>
-      </c>
-      <c r="M320" t="n">
-        <v>0</v>
-      </c>
-      <c r="N320" t="n">
-        <v>0.9728333333333333</v>
-      </c>
-      <c r="O320" t="n">
-        <v>0.02266666666666667</v>
-      </c>
-    </row>
-    <row r="321">
-      <c r="A321" t="n">
-        <v>20</v>
-      </c>
-      <c r="B321" t="n">
-        <v>10</v>
-      </c>
-      <c r="C321" t="n">
-        <v>5110</v>
-      </c>
-      <c r="D321" t="n">
-        <v>0.003913894324853229</v>
-      </c>
-      <c r="E321" t="n">
-        <v>15.884733</v>
-      </c>
-      <c r="F321" t="n">
-        <v>0.003108558317025441</v>
-      </c>
-      <c r="G321" t="n">
-        <v>30000</v>
-      </c>
-      <c r="H321" t="n">
-        <v>142</v>
-      </c>
-      <c r="I321" t="n">
-        <v>93</v>
-      </c>
-      <c r="J321" t="n">
-        <v>29765</v>
-      </c>
-      <c r="K321" t="n">
-        <v>0</v>
-      </c>
-      <c r="L321" t="n">
-        <v>0.004733333333333333</v>
-      </c>
-      <c r="M321" t="n">
-        <v>0.0031</v>
-      </c>
-      <c r="N321" t="n">
-        <v>0.9921666666666666</v>
-      </c>
-      <c r="O321" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="322">
-      <c r="A322" t="n">
-        <v>40</v>
-      </c>
-      <c r="B322" t="n">
-        <v>10</v>
-      </c>
-      <c r="C322" t="n">
-        <v>5110</v>
-      </c>
-      <c r="D322" t="n">
-        <v>0.007827788649706457</v>
-      </c>
-      <c r="E322" t="n">
-        <v>23.273367</v>
-      </c>
-      <c r="F322" t="n">
-        <v>0.004554474951076321</v>
-      </c>
-      <c r="G322" t="n">
-        <v>30000</v>
-      </c>
-      <c r="H322" t="n">
-        <v>41</v>
-      </c>
-      <c r="I322" t="n">
-        <v>5</v>
-      </c>
-      <c r="J322" t="n">
-        <v>29954</v>
-      </c>
-      <c r="K322" t="n">
-        <v>0</v>
-      </c>
-      <c r="L322" t="n">
-        <v>0.001366666666666667</v>
-      </c>
-      <c r="M322" t="n">
-        <v>0.0001666666666666667</v>
-      </c>
-      <c r="N322" t="n">
-        <v>0.9984666666666666</v>
-      </c>
-      <c r="O322" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="323">
-      <c r="A323" t="n">
-        <v>60</v>
-      </c>
-      <c r="B323" t="n">
-        <v>10</v>
-      </c>
-      <c r="C323" t="n">
-        <v>5110</v>
-      </c>
-      <c r="D323" t="n">
-        <v>0.01174168297455969</v>
-      </c>
-      <c r="E323" t="n">
-        <v>25.9887</v>
-      </c>
-      <c r="F323" t="n">
-        <v>0.005085851272015656</v>
-      </c>
-      <c r="G323" t="n">
-        <v>30000</v>
-      </c>
-      <c r="H323" t="n">
-        <v>15</v>
-      </c>
-      <c r="I323" t="n">
-        <v>0</v>
-      </c>
-      <c r="J323" t="n">
-        <v>29985</v>
-      </c>
-      <c r="K323" t="n">
-        <v>0</v>
-      </c>
-      <c r="L323" t="n">
-        <v>0.0005</v>
-      </c>
-      <c r="M323" t="n">
-        <v>0</v>
-      </c>
-      <c r="N323" t="n">
-        <v>0.9995000000000001</v>
-      </c>
-      <c r="O323" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="324">
-      <c r="A324" t="n">
-        <v>102</v>
-      </c>
-      <c r="B324" t="n">
-        <v>10</v>
-      </c>
-      <c r="C324" t="n">
-        <v>5110</v>
-      </c>
-      <c r="D324" t="n">
-        <v>0.01996086105675147</v>
-      </c>
-      <c r="E324" t="n">
-        <v>26.4037</v>
-      </c>
-      <c r="F324" t="n">
-        <v>0.005167064579256361</v>
-      </c>
-      <c r="G324" t="n">
-        <v>30000</v>
-      </c>
-      <c r="H324" t="n">
-        <v>19</v>
-      </c>
-      <c r="I324" t="n">
-        <v>0</v>
-      </c>
-      <c r="J324" t="n">
-        <v>29961</v>
-      </c>
-      <c r="K324" t="n">
-        <v>20</v>
-      </c>
-      <c r="L324" t="n">
-        <v>0.0006333333333333333</v>
-      </c>
-      <c r="M324" t="n">
-        <v>0</v>
-      </c>
-      <c r="N324" t="n">
-        <v>0.9987</v>
-      </c>
-      <c r="O324" t="n">
-        <v>0.0006666666666666666</v>
-      </c>
-    </row>
-    <row r="325">
-      <c r="A325" t="n">
-        <v>20</v>
-      </c>
-      <c r="B325" t="n">
-        <v>11</v>
-      </c>
-      <c r="C325" t="n">
-        <v>11253</v>
-      </c>
-      <c r="D325" t="n">
-        <v>0.001777303830089754</v>
-      </c>
-      <c r="E325" t="n">
-        <v>17.141133</v>
-      </c>
-      <c r="F325" t="n">
-        <v>0.001523250066648894</v>
-      </c>
-      <c r="G325" t="n">
-        <v>30000</v>
-      </c>
-      <c r="H325" t="n">
-        <v>38</v>
-      </c>
-      <c r="I325" t="n">
-        <v>51</v>
-      </c>
-      <c r="J325" t="n">
-        <v>29911</v>
-      </c>
-      <c r="K325" t="n">
-        <v>0</v>
-      </c>
-      <c r="L325" t="n">
-        <v>0.001266666666666667</v>
-      </c>
-      <c r="M325" t="n">
-        <v>0.0017</v>
-      </c>
-      <c r="N325" t="n">
-        <v>0.9970333333333333</v>
-      </c>
-      <c r="O325" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="326">
-      <c r="A326" t="n">
-        <v>20</v>
-      </c>
-      <c r="B326" t="n">
-        <v>12</v>
-      </c>
-      <c r="C326" t="n">
-        <v>24564</v>
-      </c>
-      <c r="D326" t="n">
-        <v>0.0008141996417521576</v>
-      </c>
-      <c r="E326" t="n">
-        <v>18.048667</v>
-      </c>
-      <c r="F326" t="n">
-        <v>0.0007347609102751994</v>
-      </c>
-      <c r="G326" t="n">
-        <v>30000</v>
-      </c>
-      <c r="H326" t="n">
-        <v>6</v>
-      </c>
-      <c r="I326" t="n">
-        <v>11</v>
-      </c>
-      <c r="J326" t="n">
-        <v>29983</v>
-      </c>
-      <c r="K326" t="n">
-        <v>0</v>
-      </c>
-      <c r="L326" t="n">
-        <v>0.0002</v>
-      </c>
-      <c r="M326" t="n">
-        <v>0.0003666666666666667</v>
-      </c>
-      <c r="N326" t="n">
-        <v>0.9994333333333333</v>
-      </c>
-      <c r="O326" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="327">
-      <c r="A327" t="n">
-        <v>20</v>
-      </c>
-      <c r="B327" t="n">
-        <v>13</v>
-      </c>
-      <c r="C327" t="n">
-        <v>53235</v>
-      </c>
-      <c r="D327" t="n">
-        <v>0.0003756926833849911</v>
-      </c>
-      <c r="E327" t="n">
-        <v>18.6665</v>
-      </c>
-      <c r="F327" t="n">
-        <v>0.0003506433737202968</v>
-      </c>
-      <c r="G327" t="n">
-        <v>30000</v>
-      </c>
-      <c r="H327" t="n">
-        <v>7</v>
-      </c>
-      <c r="I327" t="n">
-        <v>5</v>
-      </c>
-      <c r="J327" t="n">
-        <v>29988</v>
-      </c>
-      <c r="K327" t="n">
-        <v>0</v>
-      </c>
-      <c r="L327" t="n">
-        <v>0.0002333333333333333</v>
-      </c>
-      <c r="M327" t="n">
-        <v>0.0001666666666666667</v>
-      </c>
-      <c r="N327" t="n">
-        <v>0.9996</v>
-      </c>
-      <c r="O327" t="n">
-        <v>0</v>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:O327"/>
+  <autoFilter ref="A1:O315"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>